<commit_message>
Update: Cleaned cache files and latest changes
</commit_message>
<xml_diff>
--- a/backend/crypto_predictions_sample.xlsx
+++ b/backend/crypto_predictions_sample.xlsx
@@ -558,40 +558,40 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>71243.75780000001</v>
+        <v>80800</v>
       </c>
       <c r="E2" t="n">
-        <v>71661.5192</v>
+        <v>80214.8002</v>
       </c>
       <c r="F2" t="n">
-        <v>0.59</v>
+        <v>-0.72</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>+0.59%</t>
+          <t>-0.72%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>91.09999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>91.1%</t>
+          <t>87.7%</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904502</t>
+          <t>2026-05-05T10:00:24.994679</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -644,40 +644,40 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>71307.25380000001</v>
+        <v>80800</v>
       </c>
       <c r="E3" t="n">
-        <v>71687.3806</v>
+        <v>80367.26089999999</v>
       </c>
       <c r="F3" t="n">
-        <v>0.53</v>
+        <v>-0.54</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>+0.53%</t>
+          <t>-0.54%</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>78.09999999999999</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>78.1%</t>
+          <t>78.4%</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904563</t>
+          <t>2026-05-05T10:00:24.994748</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -730,17 +730,17 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>71146.6249</v>
+        <v>80800</v>
       </c>
       <c r="E4" t="n">
-        <v>72815.4066</v>
+        <v>82297.1997</v>
       </c>
       <c r="F4" t="n">
-        <v>2.35</v>
+        <v>1.85</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>+2.35%</t>
+          <t>+1.85%</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -749,11 +749,11 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>90.7</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>90.7%</t>
+          <t>70.4%</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904590</t>
+          <t>2026-05-05T10:00:24.994788</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -816,40 +816,40 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>71083.5775</v>
+        <v>80800</v>
       </c>
       <c r="E5" t="n">
-        <v>71033.9185</v>
+        <v>84121.27009999999</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.07000000000000001</v>
+        <v>4.11</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>+4.11%</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>72.59999999999999</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>72.6%</t>
+          <t>85.4%</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904615</t>
+          <t>2026-05-05T10:00:24.994827</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -902,30 +902,30 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>71010.1185</v>
+        <v>80800</v>
       </c>
       <c r="E6" t="n">
-        <v>71086.17999999999</v>
+        <v>82706.6422</v>
       </c>
       <c r="F6" t="n">
-        <v>0.11</v>
+        <v>2.36</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>+0.11%</t>
+          <t>+2.36%</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>62.2</v>
+        <v>60</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>62.2%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904642</t>
+          <t>2026-05-05T10:00:24.994868</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -988,17 +988,17 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3860.5986</v>
+        <v>2379.92</v>
       </c>
       <c r="E7" t="n">
-        <v>3886.0244</v>
+        <v>2394.5713</v>
       </c>
       <c r="F7" t="n">
-        <v>0.66</v>
+        <v>0.62</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>+0.66%</t>
+          <t>+0.62%</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1007,11 +1007,11 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>91.5</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>91.5%</t>
+          <t>70.9%</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904672</t>
+          <t>2026-05-05T10:00:24.994918</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1074,40 +1074,40 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3843.3633</v>
+        <v>2379.92</v>
       </c>
       <c r="E8" t="n">
-        <v>3888.759</v>
+        <v>2364.9094</v>
       </c>
       <c r="F8" t="n">
-        <v>1.18</v>
+        <v>-0.63</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>+1.18%</t>
+          <t>-0.63%</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>70</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>75.6%</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904691</t>
+          <t>2026-05-05T10:00:24.994938</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1160,40 +1160,40 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3855.128</v>
+        <v>2379.92</v>
       </c>
       <c r="E9" t="n">
-        <v>3830.5484</v>
+        <v>2386.8124</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.64</v>
+        <v>0.29</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.64%</t>
+          <t>+0.29%</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>68.40000000000001</v>
+        <v>63.7</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>68.4%</t>
+          <t>63.7%</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904712</t>
+          <t>2026-05-05T10:00:24.994957</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1246,40 +1246,40 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3842.4962</v>
+        <v>2379.92</v>
       </c>
       <c r="E10" t="n">
-        <v>4018.6815</v>
+        <v>2364.9726</v>
       </c>
       <c r="F10" t="n">
-        <v>4.59</v>
+        <v>-0.63</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>+4.59%</t>
+          <t>-0.63%</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>84.40000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>84.4%</t>
+          <t>85.9%</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904730</t>
+          <t>2026-05-05T10:00:24.994988</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1332,30 +1332,30 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3856.2162</v>
+        <v>2379.92</v>
       </c>
       <c r="E11" t="n">
-        <v>3904.3523</v>
+        <v>2383.4827</v>
       </c>
       <c r="F11" t="n">
-        <v>1.25</v>
+        <v>0.15</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>+1.25%</t>
+          <t>+0.15%</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>78.40000000000001</v>
+        <v>60</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>78.4%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904749</t>
+          <t>2026-05-05T10:00:24.995023</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1418,40 +1418,40 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>720.5725</v>
+        <v>626.63</v>
       </c>
       <c r="E12" t="n">
-        <v>715.1528</v>
+        <v>630.8951</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.75</v>
+        <v>0.68</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>+0.68%</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>75.5</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>75.5%</t>
+          <t>70.9%</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904775</t>
+          <t>2026-05-05T10:00:24.995113</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1504,30 +1504,30 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>722.5969</v>
+        <v>626.63</v>
       </c>
       <c r="E13" t="n">
-        <v>714.9207</v>
+        <v>625.3689000000001</v>
       </c>
       <c r="F13" t="n">
-        <v>-1.06</v>
+        <v>-0.2</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.06%</t>
+          <t>-0.20%</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>74.5</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>74.5%</t>
+          <t>77.4%</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904794</t>
+          <t>2026-05-05T10:00:24.995153</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1590,40 +1590,40 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>719.1113</v>
+        <v>626.63</v>
       </c>
       <c r="E14" t="n">
-        <v>718.9501</v>
+        <v>638.3392</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.02</v>
+        <v>1.87</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>+1.87%</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>75</v>
+        <v>71.8</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>71.8%</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904811</t>
+          <t>2026-05-05T10:00:24.995185</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1676,40 +1676,40 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>720.3692</v>
+        <v>626.63</v>
       </c>
       <c r="E15" t="n">
-        <v>719.7354</v>
+        <v>647.6667</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.09</v>
+        <v>3.36</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>+3.36%</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>68</v>
+        <v>84.2</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>68.0%</t>
+          <t>84.2%</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904827</t>
+          <t>2026-05-05T10:00:24.995222</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1762,40 +1762,40 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>719.8747</v>
+        <v>626.63</v>
       </c>
       <c r="E16" t="n">
-        <v>687.3972</v>
+        <v>653.8831</v>
       </c>
       <c r="F16" t="n">
-        <v>-4.51</v>
+        <v>4.35</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>-4.51%</t>
+          <t>+4.35%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>83.5</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>83.5%</t>
+          <t>83.1%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904844</t>
+          <t>2026-05-05T10:00:24.995257</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1848,40 +1848,40 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>194.08</v>
+        <v>84.69</v>
       </c>
       <c r="E17" t="n">
-        <v>192.0038</v>
+        <v>85.376</v>
       </c>
       <c r="F17" t="n">
-        <v>-1.07</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>-1.07%</t>
+          <t>+0.81%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>86.8</v>
+        <v>71</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>86.8%</t>
+          <t>71.0%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904865</t>
+          <t>2026-05-05T10:00:24.995297</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1934,40 +1934,40 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>194.0848</v>
+        <v>84.69</v>
       </c>
       <c r="E18" t="n">
-        <v>196.3473</v>
+        <v>84.2089</v>
       </c>
       <c r="F18" t="n">
-        <v>1.17</v>
+        <v>-0.57</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>+1.17%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>69.40000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>69.4%</t>
+          <t>93.8%</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904882</t>
+          <t>2026-05-05T10:00:24.995332</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2020,17 +2020,17 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>194.944</v>
+        <v>84.69</v>
       </c>
       <c r="E19" t="n">
-        <v>202.961</v>
+        <v>87.6641</v>
       </c>
       <c r="F19" t="n">
-        <v>4.11</v>
+        <v>3.51</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>+4.11%</t>
+          <t>+3.51%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2039,11 +2039,11 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>86.7</v>
+        <v>65.3</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>86.7%</t>
+          <t>65.3%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904899</t>
+          <t>2026-05-05T10:00:24.995363</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2106,40 +2106,40 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>194.8689</v>
+        <v>84.69</v>
       </c>
       <c r="E20" t="n">
-        <v>194.3514</v>
+        <v>86.6726</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.27</v>
+        <v>2.34</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>+2.34%</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>66</v>
+        <v>85.3</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>66.0%</t>
+          <t>85.3%</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904915</t>
+          <t>2026-05-05T10:00:24.995395</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2192,40 +2192,40 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>194.6326</v>
+        <v>84.69</v>
       </c>
       <c r="E21" t="n">
-        <v>187.9487</v>
+        <v>87.035</v>
       </c>
       <c r="F21" t="n">
-        <v>-3.43</v>
+        <v>2.77</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.43%</t>
+          <t>+2.77%</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>60</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>83.4%</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904935</t>
+          <t>2026-05-05T10:00:24.995437</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2278,30 +2278,30 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.6195000000000001</v>
+        <v>1.4</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6257</v>
+        <v>1.4026</v>
       </c>
       <c r="F22" t="n">
-        <v>1.01</v>
+        <v>0.18</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>+1.01%</t>
+          <t>+0.18%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>95</v>
+        <v>73.5</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>95.0%</t>
+          <t>73.5%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904957</t>
+          <t>2026-05-05T10:00:24.995482</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2364,40 +2364,40 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.617</v>
+        <v>1.4</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6175</v>
+        <v>1.3786</v>
       </c>
       <c r="F23" t="n">
-        <v>0.08</v>
+        <v>-1.53</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>+0.08%</t>
+          <t>-1.53%</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>63.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>63.3%</t>
+          <t>69.4%</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904974</t>
+          <t>2026-05-05T10:00:24.995499</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2450,40 +2450,40 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.6194</v>
+        <v>1.4</v>
       </c>
       <c r="E24" t="n">
-        <v>0.5987</v>
+        <v>1.4111</v>
       </c>
       <c r="F24" t="n">
-        <v>-3.34</v>
+        <v>0.79</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>-3.34%</t>
+          <t>+0.79%</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>89.3</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>89.3%</t>
+          <t>77.4%</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.904992</t>
+          <t>2026-05-05T10:00:24.995519</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2536,40 +2536,40 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.623</v>
+        <v>1.4</v>
       </c>
       <c r="E25" t="n">
-        <v>0.621</v>
+        <v>1.4698</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.32</v>
+        <v>4.99</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>+4.99%</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>60.8</v>
+        <v>79</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>60.8%</t>
+          <t>79.0%</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905009</t>
+          <t>2026-05-05T10:00:24.995542</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2622,40 +2622,40 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.62</v>
+        <v>1.4</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6299</v>
+        <v>1.3892</v>
       </c>
       <c r="F26" t="n">
-        <v>1.59</v>
+        <v>-0.77</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>+1.59%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>81.90000000000001</v>
+        <v>77.3</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>81.9%</t>
+          <t>77.3%</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905026</t>
+          <t>2026-05-05T10:00:24.995575</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2708,40 +2708,40 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.5787</v>
+        <v>0.2526</v>
       </c>
       <c r="E27" t="n">
-        <v>0.5819</v>
+        <v>0.2499</v>
       </c>
       <c r="F27" t="n">
-        <v>0.55</v>
+        <v>-1.07</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>+0.55%</t>
+          <t>-1.07%</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>95</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>95.0%</t>
+          <t>89.9%</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905054</t>
+          <t>2026-05-05T10:00:24.995615</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2794,17 +2794,17 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.5806</v>
+        <v>0.2526</v>
       </c>
       <c r="E28" t="n">
-        <v>0.5862000000000001</v>
+        <v>0.2551</v>
       </c>
       <c r="F28" t="n">
-        <v>0.97</v>
+        <v>1</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>+0.97%</t>
+          <t>+1.00%</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2813,11 +2813,11 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>80.40000000000001</v>
+        <v>92.5</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>80.4%</t>
+          <t>92.5%</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905072</t>
+          <t>2026-05-05T10:00:24.995648</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2880,40 +2880,40 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.5794</v>
+        <v>0.2526</v>
       </c>
       <c r="E29" t="n">
-        <v>0.5737</v>
+        <v>0.2557</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.98</v>
+        <v>1.25</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>+1.25%</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>86.5</v>
+        <v>69.2</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>86.5%</t>
+          <t>69.2%</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905090</t>
+          <t>2026-05-05T10:00:24.995678</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2966,40 +2966,40 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.5798</v>
+        <v>0.2526</v>
       </c>
       <c r="E30" t="n">
-        <v>0.5577</v>
+        <v>0.2534</v>
       </c>
       <c r="F30" t="n">
-        <v>-3.81</v>
+        <v>0.33</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>+0.33%</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>76.59999999999999</v>
+        <v>61.8</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>76.6%</t>
+          <t>61.8%</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905107</t>
+          <t>2026-05-05T10:00:24.995712</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3052,22 +3052,22 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.5828</v>
+        <v>0.2526</v>
       </c>
       <c r="E31" t="n">
-        <v>0.5826</v>
+        <v>0.2635</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.03</v>
+        <v>4.3</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>+4.30%</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I31" t="n">
@@ -3080,12 +3080,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905129</t>
+          <t>2026-05-05T10:00:24.995765</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3138,40 +3138,40 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>41.8126</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="E32" t="n">
-        <v>41.7947</v>
+        <v>9.3794</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.04</v>
+        <v>1.07</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>+1.07%</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>76.40000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>76.4%</t>
+          <t>74.5%</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905157</t>
+          <t>2026-05-05T10:00:24.995809</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3224,40 +3224,40 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>42.037</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="E33" t="n">
-        <v>41.1783</v>
+        <v>9.457599999999999</v>
       </c>
       <c r="F33" t="n">
-        <v>-2.04</v>
+        <v>1.91</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>-2.04%</t>
+          <t>+1.91%</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>93.09999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>93.1%</t>
+          <t>71.9%</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905181</t>
+          <t>2026-05-05T10:00:24.995840</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3310,40 +3310,40 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>41.9274</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="E34" t="n">
-        <v>41.711</v>
+        <v>9.6495</v>
       </c>
       <c r="F34" t="n">
-        <v>-0.52</v>
+        <v>3.98</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>+3.98%</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>86.40000000000001</v>
+        <v>68</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>86.4%</t>
+          <t>68.0%</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905199</t>
+          <t>2026-05-05T10:00:24.995871</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3396,40 +3396,40 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>41.8136</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="E35" t="n">
-        <v>40.8066</v>
+        <v>9.7393</v>
       </c>
       <c r="F35" t="n">
-        <v>-2.41</v>
+        <v>4.95</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>-2.41%</t>
+          <t>+4.95%</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>84.3</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>84.3%</t>
+          <t>65.4%</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905216</t>
+          <t>2026-05-05T10:00:24.995902</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -3482,17 +3482,17 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>41.9763</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="E36" t="n">
-        <v>42.0004</v>
+        <v>9.311999999999999</v>
       </c>
       <c r="F36" t="n">
-        <v>0.06</v>
+        <v>0.34</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>+0.06%</t>
+          <t>+0.34%</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3501,11 +3501,11 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>66.40000000000001</v>
+        <v>60</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>66.4%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905234</t>
+          <t>2026-05-05T10:00:24.995936</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -3568,30 +3568,30 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.1792</v>
+        <v>0.1116</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1807</v>
+        <v>0.1116</v>
       </c>
       <c r="F37" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>+0.84%</t>
+          <t>+0.00%</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>80.7</v>
+        <v>68.8</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>80.7%</t>
+          <t>68.8%</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905255</t>
+          <t>2026-05-05T10:00:24.995969</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -3654,17 +3654,17 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.1808</v>
+        <v>0.1116</v>
       </c>
       <c r="E38" t="n">
-        <v>0.1766</v>
+        <v>0.1097</v>
       </c>
       <c r="F38" t="n">
-        <v>-2.33</v>
+        <v>-1.66</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>-2.33%</t>
+          <t>-1.66%</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3673,11 +3673,11 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>83.59999999999999</v>
+        <v>94</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>83.6%</t>
+          <t>94.0%</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905273</t>
+          <t>2026-05-05T10:00:24.995995</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3740,40 +3740,40 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.1795</v>
+        <v>0.1116</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1874</v>
+        <v>0.1109</v>
       </c>
       <c r="F39" t="n">
-        <v>4.37</v>
+        <v>-0.59</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>+4.37%</t>
+          <t>-0.59%</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>77.09999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>77.1%</t>
+          <t>78.2%</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905289</t>
+          <t>2026-05-05T10:00:24.996027</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3826,17 +3826,17 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.1801</v>
+        <v>0.1116</v>
       </c>
       <c r="E40" t="n">
-        <v>0.1769</v>
+        <v>0.1099</v>
       </c>
       <c r="F40" t="n">
-        <v>-1.8</v>
+        <v>-1.53</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>-1.80%</t>
+          <t>-1.53%</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3845,11 +3845,11 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>77.5</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>77.5%</t>
+          <t>84.1%</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905306</t>
+          <t>2026-05-05T10:00:24.996058</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3912,40 +3912,40 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.1801</v>
+        <v>0.1116</v>
       </c>
       <c r="E41" t="n">
-        <v>0.1803</v>
+        <v>0.1089</v>
       </c>
       <c r="F41" t="n">
-        <v>0.14</v>
+        <v>-2.42</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>+0.14%</t>
+          <t>-2.42%</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>60</v>
+        <v>61.7</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>61.7%</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905322</t>
+          <t>2026-05-05T10:00:24.996088</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3998,17 +3998,17 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>8.5342</v>
+        <v>1.24</v>
       </c>
       <c r="E42" t="n">
-        <v>8.584899999999999</v>
+        <v>1.248</v>
       </c>
       <c r="F42" t="n">
-        <v>0.59</v>
+        <v>0.64</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>+0.59%</t>
+          <t>+0.64%</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4017,11 +4017,11 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>85.09999999999999</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>85.1%</t>
+          <t>86.4%</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905343</t>
+          <t>2026-05-05T10:00:24.996111</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4084,30 +4084,30 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>8.537800000000001</v>
+        <v>1.24</v>
       </c>
       <c r="E43" t="n">
-        <v>8.6204</v>
+        <v>1.2445</v>
       </c>
       <c r="F43" t="n">
-        <v>0.97</v>
+        <v>0.36</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>+0.97%</t>
+          <t>+0.36%</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>86.3</v>
+        <v>68.7</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>86.3%</t>
+          <t>68.7%</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905360</t>
+          <t>2026-05-05T10:00:24.996141</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -4170,17 +4170,17 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>8.4978</v>
+        <v>1.24</v>
       </c>
       <c r="E44" t="n">
-        <v>8.273899999999999</v>
+        <v>1.217</v>
       </c>
       <c r="F44" t="n">
-        <v>-2.63</v>
+        <v>-1.86</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>-2.63%</t>
+          <t>-1.86%</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4189,11 +4189,11 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>76.5</v>
+        <v>77.8</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>76.5%</t>
+          <t>77.8%</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905377</t>
+          <t>2026-05-05T10:00:24.996171</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -4256,17 +4256,17 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>8.5252</v>
+        <v>1.24</v>
       </c>
       <c r="E45" t="n">
-        <v>8.395200000000001</v>
+        <v>1.1816</v>
       </c>
       <c r="F45" t="n">
-        <v>-1.53</v>
+        <v>-4.71</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>-1.53%</t>
+          <t>-4.71%</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4275,11 +4275,11 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>89.0%</t>
+          <t>66.0%</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905394</t>
+          <t>2026-05-05T10:00:24.996192</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -4342,40 +4342,40 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>8.4825</v>
+        <v>1.24</v>
       </c>
       <c r="E46" t="n">
-        <v>8.1157</v>
+        <v>1.2659</v>
       </c>
       <c r="F46" t="n">
-        <v>-4.32</v>
+        <v>2.09</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>-4.32%</t>
+          <t>+2.09%</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>83.09999999999999</v>
+        <v>60.5</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>83.1%</t>
+          <t>60.5%</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905410</t>
+          <t>2026-05-05T10:00:24.996226</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -4428,40 +4428,40 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>18.5597</v>
+        <v>9.52</v>
       </c>
       <c r="E47" t="n">
-        <v>18.7382</v>
+        <v>9.4834</v>
       </c>
       <c r="F47" t="n">
-        <v>0.96</v>
+        <v>-0.38</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>+0.96%</t>
+          <t>-0.38%</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>87.2</v>
+        <v>73</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>87.2%</t>
+          <t>73.0%</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905430</t>
+          <t>2026-05-05T10:00:24.996249</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -4514,17 +4514,17 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18.5071</v>
+        <v>9.52</v>
       </c>
       <c r="E48" t="n">
-        <v>18.2254</v>
+        <v>9.453799999999999</v>
       </c>
       <c r="F48" t="n">
-        <v>-1.52</v>
+        <v>-0.7</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>-1.52%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4533,11 +4533,11 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>73.40000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>73.4%</t>
+          <t>72.8%</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905448</t>
+          <t>2026-05-05T10:00:24.996283</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -4600,30 +4600,30 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>18.5177</v>
+        <v>9.52</v>
       </c>
       <c r="E49" t="n">
-        <v>18.1179</v>
+        <v>9.501899999999999</v>
       </c>
       <c r="F49" t="n">
-        <v>-2.16</v>
+        <v>-0.19</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>-2.16%</t>
+          <t>-0.19%</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>77.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>77.2%</t>
+          <t>72.1%</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905465</t>
+          <t>2026-05-05T10:00:24.996318</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -4686,40 +4686,40 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>18.4121</v>
+        <v>9.52</v>
       </c>
       <c r="E50" t="n">
-        <v>17.5683</v>
+        <v>9.808199999999999</v>
       </c>
       <c r="F50" t="n">
-        <v>-4.58</v>
+        <v>3.03</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>-4.58%</t>
+          <t>+3.03%</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>65.3</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>65.3%</t>
+          <t>82.9%</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905483</t>
+          <t>2026-05-05T10:00:24.996344</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -4772,17 +4772,17 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>18.5566</v>
+        <v>9.52</v>
       </c>
       <c r="E51" t="n">
-        <v>18.8504</v>
+        <v>9.5969</v>
       </c>
       <c r="F51" t="n">
-        <v>1.58</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>+1.58%</t>
+          <t>+0.81%</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4791,11 +4791,11 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>74.40000000000001</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>74.4%</t>
+          <t>77.1%</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905501</t>
+          <t>2026-05-05T10:00:24.996376</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -4944,25 +4944,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>90.7</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>90.7%</t>
+          <t>70.4%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>71146.6249</v>
+        <v>80800</v>
       </c>
       <c r="G2" t="n">
-        <v>72815.4066</v>
+        <v>82297.1997</v>
       </c>
       <c r="H2" t="n">
-        <v>2.35</v>
+        <v>1.85</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>+2.35%</t>
+          <t>+1.85%</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -4974,14 +4974,14 @@
         <v>3</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M2" t="n">
-        <v>78.90000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>
@@ -4998,48 +4998,48 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>68.40000000000001</v>
+        <v>63.7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>68.4%</t>
+          <t>63.7%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>3855.128</v>
+        <v>2379.92</v>
       </c>
       <c r="G3" t="n">
-        <v>3830.5484</v>
+        <v>2386.8124</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.64</v>
+        <v>0.29</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>-0.64%</t>
+          <t>+0.29%</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M3" t="n">
-        <v>78.5</v>
+        <v>71.2</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>
@@ -5056,48 +5056,48 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>75</v>
+        <v>71.8</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>71.8%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>719.1113</v>
+        <v>626.63</v>
       </c>
       <c r="G4" t="n">
-        <v>718.9501</v>
+        <v>638.3392</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.02</v>
+        <v>1.87</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>+1.87%</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="K4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" t="n">
-        <v>3</v>
-      </c>
       <c r="M4" t="n">
-        <v>75.3</v>
+        <v>77.5</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>
@@ -5118,25 +5118,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>86.7</v>
+        <v>65.3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>86.7%</t>
+          <t>65.3%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>194.944</v>
+        <v>84.69</v>
       </c>
       <c r="G5" t="n">
-        <v>202.961</v>
+        <v>87.6641</v>
       </c>
       <c r="H5" t="n">
-        <v>4.11</v>
+        <v>3.51</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>+4.11%</t>
+          <t>+3.51%</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -5145,17 +5145,17 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>73.8</v>
+        <v>79.8</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>
@@ -5172,48 +5172,48 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>89.3</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>89.3%</t>
+          <t>77.4%</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.6194</v>
+        <v>1.4</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5987</v>
+        <v>1.4111</v>
       </c>
       <c r="H6" t="n">
-        <v>-3.34</v>
+        <v>0.79</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>-3.34%</t>
+          <t>+0.79%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="K6" t="n">
         <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" t="n">
-        <v>78.09999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>
@@ -5230,48 +5230,48 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>86.5</v>
+        <v>69.2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>86.5%</t>
+          <t>69.2%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.5794</v>
+        <v>0.2526</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5737</v>
+        <v>0.2557</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.98</v>
+        <v>1.25</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>+1.25%</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>79.7</v>
+        <v>74.7</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>
@@ -5288,48 +5288,48 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>86.40000000000001</v>
+        <v>68</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>86.4%</t>
+          <t>68.0%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>41.9274</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>41.711</v>
+        <v>9.6495</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.52</v>
+        <v>3.98</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>+3.98%</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="K8" t="n">
+        <v>4</v>
+      </c>
+      <c r="L8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" t="n">
-        <v>3</v>
-      </c>
       <c r="M8" t="n">
-        <v>81.3</v>
+        <v>68</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>
@@ -5346,48 +5346,48 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>77.09999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>77.1%</t>
+          <t>78.2%</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.1795</v>
+        <v>0.1116</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1874</v>
+        <v>0.1109</v>
       </c>
       <c r="H9" t="n">
-        <v>4.37</v>
+        <v>-0.59</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>+4.37%</t>
+          <t>-0.59%</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M9" t="n">
-        <v>75.8</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>
@@ -5408,25 +5408,25 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>76.5</v>
+        <v>77.8</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>76.5%</t>
+          <t>77.8%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>8.4978</v>
+        <v>1.24</v>
       </c>
       <c r="G10" t="n">
-        <v>8.273899999999999</v>
+        <v>1.217</v>
       </c>
       <c r="H10" t="n">
-        <v>-2.63</v>
+        <v>-1.86</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-2.63%</t>
+          <t>-1.86%</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -5438,14 +5438,14 @@
         <v>2</v>
       </c>
       <c r="L10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M10" t="n">
-        <v>84</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>
@@ -5462,29 +5462,29 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>77.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>77.2%</t>
+          <t>72.1%</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>18.5177</v>
+        <v>9.52</v>
       </c>
       <c r="G11" t="n">
-        <v>18.1179</v>
+        <v>9.501899999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>-2.16</v>
+        <v>-0.19</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>-2.16%</t>
+          <t>-0.19%</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -5496,14 +5496,14 @@
         <v>2</v>
       </c>
       <c r="L11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>75.5</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-04-13T21:03:52.905512</t>
+          <t>2026-05-05T10:00:24.996396</t>
         </is>
       </c>
     </row>

</xml_diff>